<commit_message>
Actualización automática $(date +'%d-%m-%Y %H:%M:%S')
</commit_message>
<xml_diff>
--- a/PLANTILLA_MASIVA_V2.xlsx
+++ b/PLANTILLA_MASIVA_V2.xlsx
@@ -1,37 +1,90 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abrah\OneDrive\Desktop\materiales_acumulado_app_final\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DFA70AF-F662-4606-9596-BE4978469E0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="195" yWindow="600" windowWidth="28605" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="CARGA_STOCK" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CARGA_STOCK" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+  <si>
+    <t>CODIGO AX</t>
+  </si>
+  <si>
+    <t>DESCRIPCION DEL MATERIAL</t>
+  </si>
+  <si>
+    <t>CONTRATA</t>
+  </si>
+  <si>
+    <t>BRIGADA</t>
+  </si>
+  <si>
+    <t>UNIDAD</t>
+  </si>
+  <si>
+    <t>CANTIDAD</t>
+  </si>
+  <si>
+    <t>000010136</t>
+  </si>
+  <si>
+    <t>MUFA VERTICA TERMOCONTRAIBLE</t>
+  </si>
+  <si>
+    <t>EJEMPLO_CONTRATA</t>
+  </si>
+  <si>
+    <t>LIMA B1</t>
+  </si>
+  <si>
+    <t>UNI</t>
+  </si>
+  <si>
+    <t>000018738</t>
+  </si>
+  <si>
+    <t>INVERSOR 1 A 2</t>
+  </si>
+  <si>
+    <t>HUANCAYO</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,93 +99,43 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,111 +423,73 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="45" customWidth="1"/>
+    <col min="3" max="4" width="20" customWidth="1"/>
+    <col min="5" max="6" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>CODIGO AX</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>DESCRIPCION DEL MATERIAL</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>CONTRATA</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>BRIGADA</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>UNIDAD</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>CANTIDAD</t>
-        </is>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>000010136</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>MUFA VERTICA TERMOCONTRAIBLE</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>EJEMPLO_CONTRATA</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>LIMA B1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>UNI</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
         <v>10</v>
       </c>
+      <c r="F2">
+        <v>10</v>
+      </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>000018738</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>INVERSOR 1 A 2</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>EJEMPLO_CONTRATA</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>HUANCAYO B2</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>UNI</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: dar soporte nativo al nuevo excel Formato de Diario de Embarque (Carso) con extraccion de cabeceras automaticas
</commit_message>
<xml_diff>
--- a/PLANTILLA_MASIVA_V2.xlsx
+++ b/PLANTILLA_MASIVA_V2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abrah\OneDrive\Desktop\PROYECTOS_INSIGHT\materiales_acumulado_app_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EEA59CF-C8DC-45DB-8A21-895D28E273F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B45142-FB80-4767-870A-098522211503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="705" yWindow="0" windowWidth="28605" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CARGA_STOCK" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="28">
   <si>
     <t>CODIGO AX</t>
   </si>
@@ -53,21 +53,6 @@
     <t>CANTIDAD</t>
   </si>
   <si>
-    <t>ECYTEL</t>
-  </si>
-  <si>
-    <t>LIMA B4</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>LIMA B6</t>
-  </si>
-  <si>
-    <t>Unidad</t>
-  </si>
-  <si>
     <r>
       <t>COMERCIAL</t>
     </r>
@@ -82,221 +67,77 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">SPLITER 1 X 4 </t>
+    <t>CONMATEL SAC</t>
   </si>
   <si>
-    <t>SPLITER 1 X 8</t>
+    <t>LIMA B3</t>
   </si>
   <si>
-    <t>PREFORMADO VERDE</t>
+    <t>unidad</t>
   </si>
   <si>
-    <t xml:space="preserve">CABLE 96 MM </t>
+    <t xml:space="preserve">CABLE DE 96 SM </t>
   </si>
   <si>
-    <t xml:space="preserve">CABLE 96 SM </t>
+    <t xml:space="preserve">CABLE DE 144 HILOS </t>
   </si>
   <si>
-    <t xml:space="preserve">MUFA DOMO </t>
+    <t xml:space="preserve">CABLE DUAL 100 MTS </t>
   </si>
   <si>
-    <t xml:space="preserve">MUFA HORIZONTAL </t>
+    <t xml:space="preserve">CABLE DUAL 150 MTS </t>
   </si>
   <si>
-    <t xml:space="preserve">PREFORMADO AZUL </t>
+    <t xml:space="preserve">CABLE DUAL 200 MTS </t>
   </si>
   <si>
-    <t>PREFORMADO NARANJA</t>
+    <t>LIMA B7</t>
   </si>
   <si>
-    <t>AISLADOR</t>
+    <t>HEBILLA DE 5/8</t>
   </si>
   <si>
-    <t>CLEVIS</t>
+    <t>metros</t>
   </si>
   <si>
-    <t xml:space="preserve">CINTA BANDIT </t>
+    <t>CINTA BANDIT 5/8</t>
   </si>
   <si>
-    <t>CABLE FO ANTIROEDOR ADSS144G.652D-250 HT</t>
+    <t xml:space="preserve">HUXBOX - NEGRO </t>
   </si>
   <si>
-    <t>1043110 - C OADSSI0 CX87 ATE DL 48SMF BK WRL 6000M (DESMONTADO)</t>
+    <t xml:space="preserve">FAT FINAL </t>
   </si>
   <si>
-    <t>1043105 - C OADSS60 CX87 DDE DL 48SMF BK WRL (DESMONTADO)</t>
+    <t xml:space="preserve">HUBBOX - BLANCO </t>
   </si>
   <si>
-    <t>CABLE FO 48H SM400 MONOMODO D/CANTIHIELO</t>
+    <t>LIMA B9</t>
   </si>
   <si>
-    <t>SPLITTER SPL9102-PLC-1016M 45200687 HW</t>
+    <t xml:space="preserve">CABLE DE 48 SM </t>
   </si>
   <si>
-    <t>CIERRE DE EMPALME RHS04-FOSC-144FM6B</t>
+    <t xml:space="preserve">REDUCTOR </t>
   </si>
   <si>
-    <t>CIERRE EMPALME SSC2823-SH-8B 14261249 HW</t>
+    <t>HEBUILLA DE 5/8</t>
   </si>
   <si>
-    <t>CABLE MPO PRECO EOCPAPC43 - MPO 300M</t>
+    <t xml:space="preserve">CLOSSURE DE 96 </t>
   </si>
   <si>
-    <t>CABLE PRECO DISTRIBUCION DUAL CORE E0SDC056 - DLC 150M</t>
+    <t xml:space="preserve">MUFA DE 144 HILOS </t>
   </si>
   <si>
-    <t>CABLE PRECO DISTRIBUCION DUAL CORE E0SDC055 - DLC 100M</t>
-  </si>
-  <si>
-    <t>ORDENADOR DE FIBRA FAT ITC3105</t>
-  </si>
-  <si>
-    <t>CIERRE DE EMPALME FAT SSC2816-SM-9</t>
-  </si>
-  <si>
-    <t>CIERRE DE EMPALME FAT SSC2816-SM-11U</t>
-  </si>
-  <si>
-    <t>MPO PIGTAIL SS-OP-MPO-SC-S-1.5</t>
-  </si>
-  <si>
-    <t>CIERRE DE EMPALME XBOX SSC2807-FX-12-B</t>
-  </si>
-  <si>
-    <t>CIERRE DE EMPALMETE HUBBOX SSC2823-SH-16-B</t>
-  </si>
-  <si>
-    <t>CIERRE DE EMPALME FAT 8 SALIDAS 14260813</t>
-  </si>
-  <si>
-    <t>CIERRE EMPALME HUBBOX 8O PRECON 52343655</t>
-  </si>
-  <si>
-    <t>CIERRE DE EMPALME FAT 9 SALIDAS 14260812</t>
-  </si>
-  <si>
-    <t>C OADSSI0 CX87 ATE DL 48SMF BK WRL 6000M</t>
-  </si>
-  <si>
-    <t>CABLE ADSS-144 HILOS SM - G.652D SPAN 250 M</t>
-  </si>
-  <si>
-    <t>PIGTAIL-SC/APC SM G.657A2-0.9MM-1M</t>
-  </si>
-  <si>
-    <t>CIERRE DE EMPALME 144H - FOSC-260R-B106-#07</t>
-  </si>
-  <si>
-    <t>HERRAJE ORDENADOR DE RESERVA PARA FAT</t>
-  </si>
-  <si>
-    <t>FAT EVEN 8 SALIDAS</t>
-  </si>
-  <si>
-    <t>PRE-CONECTORIZADO DE DISTRIBUCION 250 M</t>
-  </si>
-  <si>
-    <t>PRE-CONECTORIZADO DE DISTRIBUCION 150 M</t>
-  </si>
-  <si>
-    <t>PRE-CONECTORIZADO DE DISTRIBUCION 100 M</t>
-  </si>
-  <si>
-    <t>PRE-CONECTORIZADO DE DISTRIBUCION 80 M</t>
-  </si>
-  <si>
-    <t>PRE-CONECTORIZADO DE DISTRIBUCION 50 M</t>
-  </si>
-  <si>
-    <t>PRE-CONECTORIZADO DE DISTRIBUCION 5 M</t>
-  </si>
-  <si>
-    <t>CAJA DE PISO 8 SALIDAS</t>
-  </si>
-  <si>
-    <t>CLOSSURE 96 CORES 6 OUTPUTS</t>
-  </si>
-  <si>
-    <t>CABLE FO 24F-SM ANTIROEDOR 69199 24</t>
-  </si>
-  <si>
-    <t>C OADSS85 CX87 DDE DL 24SMF BK WRL</t>
-  </si>
-  <si>
-    <t>FDT O CAJA DE 1ER NIVEL 9 SAL.</t>
-  </si>
-  <si>
-    <t>DOME CLOSSURE 48/24/12 CORES</t>
-  </si>
-  <si>
-    <t>SPL 1:4 FAT PIGTAIL SC/APC</t>
-  </si>
-  <si>
-    <t>CAJA PRECON. 8 SALIDAS INCL. KIT MO</t>
-  </si>
-  <si>
-    <t>SPL 1:8 PLC SIN CONECTOR</t>
-  </si>
-  <si>
-    <t>C OADSS60 CX87 DDE DL 48SMF BK WRL</t>
-  </si>
-  <si>
-    <t>KIT DE HERRAJE DE RETENCION SPAN 100 M - DIAM 13.3 MM (SOLO PREFORMADO)</t>
-  </si>
-  <si>
-    <t>CABLE 96F-SM ANTIROEDOR 69199 96 1 AM</t>
-  </si>
-  <si>
-    <t>CABLE ADSS 4000N (68186) 96 HILOS F.O.MM</t>
-  </si>
-  <si>
-    <t>KIT DE SELLADO PARA PUERTO OVAL ABIERTO CON RIEL</t>
-  </si>
-  <si>
-    <t>CABLE ADSS 4000N (69186) 48 HILOS F.O.SM</t>
-  </si>
-  <si>
-    <t>TERMINAL MST-08M-NN-U250-B 8PTS DLX 250M</t>
-  </si>
-  <si>
-    <t>SPLITTER FIST-FSASA3-SC-132-1P-S 1:32 SC</t>
-  </si>
-  <si>
-    <t>CABLE ADSS 4000N (69186) 24 HILOS F.O.SM</t>
-  </si>
-  <si>
-    <t>CABLE ADSS 4000N (69186) 96 HILOS F.O.SM</t>
-  </si>
-  <si>
-    <t>CABLE FO 8 SC/APC 453191-003</t>
-  </si>
-  <si>
-    <t>CIERRE DE EMPALME TIPO DOMO CAM-JB-102A-8P FOSC (4 BANDEJAS + MANGA OVAL Y CIRCULAR + 96 PROT EMPALME + SOPORTE)</t>
-  </si>
-  <si>
-    <t>REMATE PREFORMADO PARA CABLE 1/2 AZUL</t>
-  </si>
-  <si>
-    <t>REMATE PREFORMADO PARA CABLE 1/2 NARANJA</t>
-  </si>
-  <si>
-    <t>AISLADOR TIPO CARRETE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HERRAJE DE TENSION TIPO D </t>
-  </si>
-  <si>
-    <t xml:space="preserve">HEBILLA 5/8 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLEJE DE ACERO 5/8 </t>
+    <t>MPO DE 300</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -336,8 +177,12 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -352,12 +197,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor rgb="FF000000"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -380,11 +237,107 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -404,15 +357,29 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -725,7 +692,7 @@
     <col min="6" max="6" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -742,1807 +709,1040 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
+        <v>145</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="10">
+        <v>300</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="11">
+        <v>6983</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="10">
+        <v>150</v>
+      </c>
+      <c r="F3" s="12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="5">
-        <v>15132</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="4" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="11">
+        <v>10368</v>
+      </c>
+      <c r="B4" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="C4" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="5">
-        <v>1500</v>
-      </c>
-      <c r="F2" s="5" t="s">
+      <c r="D4" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="10">
+        <v>1</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="11">
+        <v>10369</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="10">
+        <v>1</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="11">
+        <v>10370</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="10">
+        <v>1</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="11">
+        <v>145</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="10">
+        <v>300</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="15">
+        <v>1124</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="18">
+        <v>60</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="15">
+        <v>1125</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="13">
+        <v>60</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="11">
+        <v>6983</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="13">
+        <v>300</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="21">
+        <v>10361</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="10">
+        <v>1</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="11">
+        <v>10365</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="10">
+        <v>1</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="14">
+        <v>10368</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="10">
+        <v>1</v>
+      </c>
+      <c r="F13" s="22" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="11">
+        <v>10369</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="23">
+        <v>1</v>
+      </c>
+      <c r="F14" s="22" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="11">
+        <v>10370</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="23">
+        <v>1</v>
+      </c>
+      <c r="F15" s="22" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="14">
+        <v>10893</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="23">
+        <v>1</v>
+      </c>
+      <c r="F16" s="22" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="24">
+        <v>145</v>
+      </c>
+      <c r="B17" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="23">
+        <v>300</v>
+      </c>
+      <c r="F17" s="26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="27">
+        <v>545</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="10">
+        <v>300</v>
+      </c>
+      <c r="F18" s="29" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="11">
+        <v>961</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E19" s="10">
+        <v>3</v>
+      </c>
+      <c r="F19" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G2" s="6"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="7">
-        <v>14647</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="8" t="s">
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="28">
+        <v>1124</v>
+      </c>
+      <c r="B20" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="D20" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="7">
-        <v>366</v>
-      </c>
-      <c r="F3" s="7" t="s">
+      <c r="E20" s="10">
+        <v>32</v>
+      </c>
+      <c r="F20" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="9"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="7">
-        <v>14646</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="8" t="s">
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="27">
+        <v>1125</v>
+      </c>
+      <c r="B21" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="D21" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="E21" s="10">
+        <v>30</v>
+      </c>
+      <c r="F21" s="25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="11">
+        <v>5797</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D22" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="7">
-        <v>946</v>
-      </c>
-      <c r="F4" s="7" t="s">
+      <c r="E22" s="23">
+        <v>1</v>
+      </c>
+      <c r="F22" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="9"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
-        <v>14183</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="4" t="s">
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="11">
+        <v>6979</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="5">
-        <v>78</v>
-      </c>
-      <c r="F5" s="5" t="s">
+      <c r="E23" s="10">
+        <v>1</v>
+      </c>
+      <c r="F23" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="6"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="5">
-        <v>14183</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="4" t="s">
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="11">
+        <v>6983</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D24" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="5">
-        <v>204</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G6" s="6"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
-        <v>12172</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="E24" s="10">
+        <v>76</v>
+      </c>
+      <c r="F24" s="29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="11">
+        <v>10368</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D25" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="5">
+      <c r="E25" s="10">
+        <v>1</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="14">
+        <v>10369</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E26" s="10">
+        <v>1</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="14">
+        <v>10371</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E27" s="10">
         <v>2</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F27" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="G7" s="6"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="5">
-        <v>11292</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="5">
-        <v>14</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G8" s="6"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="5">
-        <v>10893</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="5">
-        <v>2</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G9" s="6"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="5">
-        <v>10371</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" s="5">
-        <v>12</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G10" s="6"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="5">
-        <v>10369</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" s="5">
-        <v>1</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="G11" s="6"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="5">
-        <v>10368</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="5">
-        <v>31</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="G12" s="6"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="5">
-        <v>10367</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13" s="5">
-        <v>10</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G13" s="6"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="5">
-        <v>10365</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" s="5">
-        <v>7</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G14" s="6"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="5">
-        <v>10364</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" s="5">
-        <v>7</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="G15" s="6"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="5">
-        <v>10363</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E16" s="5">
-        <v>9</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G16" s="6"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="5">
-        <v>10362</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E17" s="5">
-        <v>2</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="G17" s="6"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="5">
-        <v>10361</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E18" s="5">
-        <v>7</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="G18" s="6"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="5">
-        <v>9201</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E19" s="5">
-        <v>3</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="G19" s="6"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="7">
-        <v>9200</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E20" s="7">
-        <v>7</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="G20" s="9"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="5">
-        <v>9199</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E21" s="5">
-        <v>6</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="G21" s="6"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="5">
-        <v>9173</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E22" s="5">
-        <v>191</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="G22" s="6"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="5">
-        <v>9173</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E23" s="5">
-        <v>1</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="G23" s="6"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="5">
-        <v>6983</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E24" s="5">
-        <v>1000</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="G24" s="6"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="5">
-        <v>6983</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E25" s="5">
-        <v>202</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="G25" s="6"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="5">
-        <v>6983</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E26" s="5">
-        <v>158</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="G26" s="6"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="5">
-        <v>6983</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E27" s="5">
-        <v>89</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="G27" s="6"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="5">
-        <v>6983</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E28" s="5">
-        <v>150</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="G28" s="6"/>
+      <c r="A28" s="5"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="6"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="5">
-        <v>6982</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E29" s="5">
-        <v>7</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>44</v>
-      </c>
+      <c r="A29" s="5"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
       <c r="G29" s="6"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="5">
-        <v>6979</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E30" s="5">
-        <v>15</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>45</v>
-      </c>
+      <c r="A30" s="5"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
       <c r="G30" s="6"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="5">
-        <v>6973</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E31" s="5">
-        <v>2</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>46</v>
-      </c>
+      <c r="A31" s="5"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
       <c r="G31" s="6"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="5">
-        <v>6972</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E32" s="5">
-        <v>1</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>47</v>
-      </c>
+      <c r="A32" s="5"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
       <c r="G32" s="6"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="5">
-        <v>6971</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E33" s="5">
-        <v>19</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>48</v>
-      </c>
+      <c r="A33" s="5"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
       <c r="G33" s="6"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="5">
-        <v>6970</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E34" s="5">
-        <v>5</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>49</v>
-      </c>
+      <c r="A34" s="5"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
       <c r="G34" s="6"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="5">
-        <v>6969</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E35" s="5">
-        <v>6</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>50</v>
-      </c>
+      <c r="A35" s="5"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
       <c r="G35" s="6"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="5">
-        <v>6968</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E36" s="5">
-        <v>5</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>51</v>
-      </c>
+      <c r="A36" s="5"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
       <c r="G36" s="6"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="5">
-        <v>6967</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E37" s="5">
-        <v>8</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>52</v>
-      </c>
+      <c r="A37" s="5"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
       <c r="G37" s="6"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="5">
-        <v>6966</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E38" s="5">
-        <v>8</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>53</v>
-      </c>
+      <c r="A38" s="5"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
       <c r="G38" s="6"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="5">
-        <v>6384</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E39" s="5">
-        <v>6</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>54</v>
-      </c>
+      <c r="A39" s="5"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5"/>
       <c r="G39" s="6"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="5">
-        <v>5797</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E40" s="5">
-        <v>37</v>
-      </c>
-      <c r="F40" s="5" t="s">
-        <v>55</v>
-      </c>
+      <c r="A40" s="5"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
       <c r="G40" s="6"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="5">
-        <v>5725</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D41" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E41" s="5">
-        <v>500</v>
-      </c>
-      <c r="F41" s="5" t="s">
-        <v>56</v>
-      </c>
+      <c r="A41" s="5"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
       <c r="G41" s="6"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="5">
-        <v>5725</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E42" s="5">
-        <v>500</v>
-      </c>
-      <c r="F42" s="5" t="s">
-        <v>56</v>
-      </c>
+      <c r="A42" s="5"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
       <c r="G42" s="6"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="5">
-        <v>5608</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D43" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E43" s="5">
-        <v>523</v>
-      </c>
-      <c r="F43" s="5" t="s">
-        <v>57</v>
-      </c>
+      <c r="A43" s="5"/>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
       <c r="G43" s="6"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="5">
-        <v>5590</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E44" s="5">
-        <v>10</v>
-      </c>
-      <c r="F44" s="5" t="s">
-        <v>58</v>
-      </c>
+      <c r="A44" s="5"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
       <c r="G44" s="6"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="5">
-        <v>5589</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D45" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E45" s="5">
-        <v>6</v>
-      </c>
-      <c r="F45" s="5" t="s">
-        <v>59</v>
-      </c>
+      <c r="A45" s="5"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
       <c r="G45" s="6"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="5">
-        <v>5588</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D46" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E46" s="5">
-        <v>8</v>
-      </c>
-      <c r="F46" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="G46" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="A46" s="5"/>
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="5"/>
+      <c r="F46" s="5"/>
+      <c r="G46" s="6"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="5">
-        <v>5587</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E47" s="5">
-        <v>7</v>
-      </c>
-      <c r="F47" s="5" t="s">
-        <v>61</v>
-      </c>
+      <c r="A47" s="5"/>
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="5"/>
+      <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
       <c r="G47" s="6"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="5">
-        <v>5586</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E48" s="5">
-        <v>7</v>
-      </c>
-      <c r="F48" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="G48" s="6" t="s">
-        <v>12</v>
-      </c>
+      <c r="A48" s="5"/>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="6"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="5">
-        <v>5567</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D49" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E49" s="5">
-        <v>1130</v>
-      </c>
-      <c r="F49" s="5" t="s">
-        <v>63</v>
-      </c>
+      <c r="A49" s="5"/>
+      <c r="B49" s="4"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
       <c r="G49" s="6"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="5">
-        <v>5504</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D50" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E50" s="5">
-        <v>60</v>
-      </c>
-      <c r="F50" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="G50" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="A50" s="5"/>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="5"/>
+      <c r="F50" s="5"/>
+      <c r="G50" s="6"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="5">
-        <v>4286</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D51" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E51" s="5">
-        <v>1000</v>
-      </c>
-      <c r="F51" s="5" t="s">
-        <v>65</v>
-      </c>
+      <c r="A51" s="5"/>
+      <c r="B51" s="4"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
       <c r="G51" s="6"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="5">
-        <v>3438</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D52" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E52" s="5">
-        <v>1018</v>
-      </c>
-      <c r="F52" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="G52" s="6" t="s">
-        <v>14</v>
-      </c>
+      <c r="A52" s="5"/>
+      <c r="B52" s="4"/>
+      <c r="C52" s="4"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="6"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="5">
-        <v>3438</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D53" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E53" s="5">
-        <v>603</v>
-      </c>
-      <c r="F53" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="G53" s="6" t="s">
-        <v>14</v>
-      </c>
+      <c r="A53" s="5"/>
+      <c r="B53" s="4"/>
+      <c r="C53" s="4"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
+      <c r="F53" s="5"/>
+      <c r="G53" s="6"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="5">
-        <v>3438</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D54" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E54" s="5">
-        <v>300</v>
-      </c>
-      <c r="F54" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="G54" s="6" t="s">
-        <v>14</v>
-      </c>
+      <c r="A54" s="5"/>
+      <c r="B54" s="4"/>
+      <c r="C54" s="4"/>
+      <c r="D54" s="5"/>
+      <c r="E54" s="5"/>
+      <c r="F54" s="5"/>
+      <c r="G54" s="6"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="5">
-        <v>1093</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D55" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E55" s="5">
-        <v>10</v>
-      </c>
-      <c r="F55" s="5" t="s">
-        <v>67</v>
-      </c>
+      <c r="A55" s="5"/>
+      <c r="B55" s="4"/>
+      <c r="C55" s="4"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
       <c r="G55" s="6"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="5">
-        <v>545</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D56" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E56" s="5">
-        <v>1000</v>
-      </c>
-      <c r="F56" s="5" t="s">
-        <v>68</v>
-      </c>
+      <c r="A56" s="5"/>
+      <c r="B56" s="4"/>
+      <c r="C56" s="4"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
       <c r="G56" s="6"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="5">
-        <v>545</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D57" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E57" s="5">
-        <v>1000</v>
-      </c>
-      <c r="F57" s="5" t="s">
-        <v>68</v>
-      </c>
+      <c r="A57" s="5"/>
+      <c r="B57" s="4"/>
+      <c r="C57" s="4"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
       <c r="G57" s="6"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="5">
-        <v>377</v>
-      </c>
-      <c r="B58" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D58" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E58" s="5">
-        <v>1</v>
-      </c>
-      <c r="F58" s="5" t="s">
-        <v>69</v>
-      </c>
+      <c r="A58" s="5"/>
+      <c r="B58" s="4"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="5"/>
       <c r="G58" s="6"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" s="5">
-        <v>373</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D59" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E59" s="5">
-        <v>1</v>
-      </c>
-      <c r="F59" s="5" t="s">
-        <v>70</v>
-      </c>
+      <c r="A59" s="5"/>
+      <c r="B59" s="4"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
+      <c r="F59" s="5"/>
       <c r="G59" s="6"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="5">
-        <v>232</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C60" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D60" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E60" s="5">
-        <v>78</v>
-      </c>
-      <c r="F60" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="G60" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="A60" s="5"/>
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
+      <c r="F60" s="5"/>
+      <c r="G60" s="6"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="5">
-        <v>232</v>
-      </c>
-      <c r="B61" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C61" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D61" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E61" s="5">
-        <v>29</v>
-      </c>
-      <c r="F61" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="G61" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="A61" s="5"/>
+      <c r="B61" s="4"/>
+      <c r="C61" s="4"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="6"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="5">
-        <v>232</v>
-      </c>
-      <c r="B62" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C62" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D62" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E62" s="5">
-        <v>120</v>
-      </c>
-      <c r="F62" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="G62" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="A62" s="5"/>
+      <c r="B62" s="4"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="5"/>
+      <c r="F62" s="5"/>
+      <c r="G62" s="6"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="5">
-        <v>232</v>
-      </c>
-      <c r="B63" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C63" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D63" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E63" s="5">
-        <v>12</v>
-      </c>
-      <c r="F63" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="G63" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="A63" s="5"/>
+      <c r="B63" s="4"/>
+      <c r="C63" s="4"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="5"/>
+      <c r="F63" s="5"/>
+      <c r="G63" s="6"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" s="5">
-        <v>145</v>
-      </c>
-      <c r="B64" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C64" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D64" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E64" s="5">
-        <v>750</v>
-      </c>
-      <c r="F64" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="G64" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="A64" s="5"/>
+      <c r="B64" s="4"/>
+      <c r="C64" s="4"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="G64" s="6"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" s="5">
-        <v>145</v>
-      </c>
-      <c r="B65" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C65" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D65" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E65" s="5">
-        <v>1000</v>
-      </c>
-      <c r="F65" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="G65" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="A65" s="5"/>
+      <c r="B65" s="4"/>
+      <c r="C65" s="4"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="5"/>
+      <c r="F65" s="5"/>
+      <c r="G65" s="6"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" s="5">
-        <v>145</v>
-      </c>
-      <c r="B66" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C66" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D66" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E66" s="5">
-        <v>455</v>
-      </c>
-      <c r="F66" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="G66" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="A66" s="5"/>
+      <c r="B66" s="4"/>
+      <c r="C66" s="4"/>
+      <c r="D66" s="5"/>
+      <c r="E66" s="5"/>
+      <c r="F66" s="5"/>
+      <c r="G66" s="6"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" s="5">
-        <v>7</v>
-      </c>
-      <c r="B67" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C67" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D67" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E67" s="5">
-        <v>7</v>
-      </c>
-      <c r="F67" s="5" t="s">
-        <v>73</v>
-      </c>
+      <c r="A67" s="5"/>
+      <c r="B67" s="4"/>
+      <c r="C67" s="4"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
       <c r="G67" s="6"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="5">
-        <v>9276</v>
-      </c>
-      <c r="B68" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C68" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D68" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E68" s="5">
-        <v>2</v>
-      </c>
-      <c r="F68" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="G68" s="6" t="s">
-        <v>16</v>
-      </c>
+      <c r="A68" s="5"/>
+      <c r="B68" s="4"/>
+      <c r="C68" s="4"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
+      <c r="G68" s="6"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" s="5">
-        <v>9277</v>
-      </c>
-      <c r="B69" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C69" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D69" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E69" s="5">
-        <v>2</v>
-      </c>
-      <c r="F69" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G69" s="6" t="s">
-        <v>17</v>
-      </c>
+      <c r="A69" s="5"/>
+      <c r="B69" s="4"/>
+      <c r="C69" s="4"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
+      <c r="G69" s="6"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" s="5">
-        <v>3412</v>
-      </c>
-      <c r="B70" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C70" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D70" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E70" s="5">
-        <v>10</v>
-      </c>
-      <c r="F70" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="G70" s="6" t="s">
-        <v>18</v>
-      </c>
+      <c r="A70" s="5"/>
+      <c r="B70" s="4"/>
+      <c r="C70" s="4"/>
+      <c r="D70" s="5"/>
+      <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
+      <c r="G70" s="6"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="5">
-        <v>3413</v>
-      </c>
-      <c r="B71" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C71" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D71" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E71" s="5">
-        <v>10</v>
-      </c>
-      <c r="F71" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="G71" s="6" t="s">
-        <v>19</v>
-      </c>
+      <c r="A71" s="5"/>
+      <c r="B71" s="4"/>
+      <c r="C71" s="4"/>
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="6"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" s="5">
-        <v>1009</v>
-      </c>
-      <c r="B72" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C72" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D72" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E72" s="5">
-        <v>10</v>
-      </c>
-      <c r="F72" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="G72" s="6" t="s">
-        <v>20</v>
-      </c>
+      <c r="A72" s="5"/>
+      <c r="B72" s="4"/>
+      <c r="C72" s="4"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="5"/>
+      <c r="F72" s="5"/>
+      <c r="G72" s="6"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A73" s="5">
-        <v>1078</v>
-      </c>
-      <c r="B73" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C73" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D73" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E73" s="5">
-        <v>10</v>
-      </c>
-      <c r="F73" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="G73" s="6" t="s">
-        <v>21</v>
-      </c>
+      <c r="A73" s="5"/>
+      <c r="B73" s="4"/>
+      <c r="C73" s="4"/>
+      <c r="D73" s="5"/>
+      <c r="E73" s="5"/>
+      <c r="F73" s="5"/>
+      <c r="G73" s="6"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A74" s="5">
-        <v>1124</v>
-      </c>
-      <c r="B74" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C74" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D74" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E74" s="5">
-        <v>20</v>
-      </c>
-      <c r="F74" s="5" t="s">
-        <v>79</v>
-      </c>
+      <c r="A74" s="5"/>
+      <c r="B74" s="4"/>
+      <c r="C74" s="4"/>
+      <c r="D74" s="5"/>
+      <c r="E74" s="5"/>
+      <c r="F74" s="5"/>
       <c r="G74" s="6"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" s="5">
-        <v>1125</v>
-      </c>
-      <c r="B75" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C75" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D75" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E75" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="F75" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="G75" s="6" t="s">
-        <v>22</v>
-      </c>
+      <c r="A75" s="5"/>
+      <c r="B75" s="4"/>
+      <c r="C75" s="4"/>
+      <c r="D75" s="5"/>
+      <c r="E75" s="5"/>
+      <c r="F75" s="5"/>
+      <c r="G75" s="6"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" s="5">
-        <v>9276</v>
-      </c>
-      <c r="B76" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C76" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D76" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E76" s="5">
-        <v>2</v>
-      </c>
-      <c r="F76" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="G76" s="6" t="s">
-        <v>16</v>
-      </c>
+      <c r="A76" s="5"/>
+      <c r="B76" s="4"/>
+      <c r="C76" s="4"/>
+      <c r="D76" s="5"/>
+      <c r="E76" s="5"/>
+      <c r="F76" s="5"/>
+      <c r="G76" s="6"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A77" s="5">
-        <v>9277</v>
-      </c>
-      <c r="B77" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C77" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D77" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E77" s="5">
-        <v>2</v>
-      </c>
-      <c r="F77" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G77" s="6" t="s">
-        <v>17</v>
-      </c>
+      <c r="A77" s="5"/>
+      <c r="B77" s="4"/>
+      <c r="C77" s="4"/>
+      <c r="D77" s="5"/>
+      <c r="E77" s="5"/>
+      <c r="F77" s="5"/>
+      <c r="G77" s="6"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A78" s="5">
-        <v>3412</v>
-      </c>
-      <c r="B78" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C78" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D78" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E78" s="5">
-        <v>10</v>
-      </c>
-      <c r="F78" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="G78" s="6" t="s">
-        <v>18</v>
-      </c>
+      <c r="A78" s="5"/>
+      <c r="B78" s="4"/>
+      <c r="C78" s="4"/>
+      <c r="D78" s="5"/>
+      <c r="E78" s="5"/>
+      <c r="F78" s="5"/>
+      <c r="G78" s="6"/>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A79" s="5">
-        <v>3413</v>
-      </c>
-      <c r="B79" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C79" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D79" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E79" s="5">
-        <v>10</v>
-      </c>
-      <c r="F79" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="G79" s="6" t="s">
-        <v>19</v>
-      </c>
+      <c r="A79" s="5"/>
+      <c r="B79" s="4"/>
+      <c r="C79" s="4"/>
+      <c r="D79" s="5"/>
+      <c r="E79" s="5"/>
+      <c r="F79" s="5"/>
+      <c r="G79" s="6"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A80" s="5">
-        <v>1009</v>
-      </c>
-      <c r="B80" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C80" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D80" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E80" s="5">
-        <v>10</v>
-      </c>
-      <c r="F80" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="G80" s="6" t="s">
-        <v>20</v>
-      </c>
+      <c r="A80" s="5"/>
+      <c r="B80" s="4"/>
+      <c r="C80" s="4"/>
+      <c r="D80" s="5"/>
+      <c r="E80" s="5"/>
+      <c r="F80" s="5"/>
+      <c r="G80" s="6"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A81" s="5">
-        <v>1078</v>
-      </c>
-      <c r="B81" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C81" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D81" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E81" s="5">
-        <v>10</v>
-      </c>
-      <c r="F81" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="G81" s="6" t="s">
-        <v>21</v>
-      </c>
+      <c r="A81" s="5"/>
+      <c r="B81" s="4"/>
+      <c r="C81" s="4"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="5"/>
+      <c r="F81" s="5"/>
+      <c r="G81" s="6"/>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A82" s="5">
-        <v>1124</v>
-      </c>
-      <c r="B82" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C82" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D82" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E82" s="5">
-        <v>20</v>
-      </c>
-      <c r="F82" s="5" t="s">
-        <v>79</v>
-      </c>
+      <c r="A82" s="5"/>
+      <c r="B82" s="4"/>
+      <c r="C82" s="4"/>
+      <c r="D82" s="5"/>
+      <c r="E82" s="5"/>
+      <c r="F82" s="5"/>
       <c r="G82" s="6"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A83" s="5">
-        <v>1125</v>
-      </c>
-      <c r="B83" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C83" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D83" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E83" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="F83" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="G83" s="6" t="s">
-        <v>22</v>
-      </c>
+      <c r="A83" s="5"/>
+      <c r="B83" s="4"/>
+      <c r="C83" s="4"/>
+      <c r="D83" s="5"/>
+      <c r="E83" s="5"/>
+      <c r="F83" s="5"/>
+      <c r="G83" s="6"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A84" s="5">
-        <v>5504</v>
-      </c>
-      <c r="B84" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C84" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D84" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E84" s="5">
-        <v>60</v>
-      </c>
-      <c r="F84" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="G84" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="A84" s="5"/>
+      <c r="B84" s="4"/>
+      <c r="C84" s="4"/>
+      <c r="D84" s="5"/>
+      <c r="E84" s="5"/>
+      <c r="F84" s="5"/>
+      <c r="G84" s="6"/>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="2"/>

</xml_diff>